<commit_message>
UPDATED ALL DATASETS including FRS, Annual ACS data, not environmental data
</commit_message>
<xml_diff>
--- a/inst/testdata/registryid/frs_testpoints_10.xlsx
+++ b/inst/testdata/registryid/frs_testpoints_10.xlsx
@@ -371,7 +371,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>110040410882</v>
+        <v>110040663047</v>
       </c>
     </row>
     <row r="3">
@@ -379,7 +379,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>110070352769</v>
+        <v>110070353219</v>
       </c>
     </row>
     <row r="4">
@@ -387,7 +387,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>110040598724</v>
+        <v>110040784933</v>
       </c>
     </row>
     <row r="5">
@@ -395,7 +395,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>110051768379</v>
+        <v>110071956718</v>
       </c>
     </row>
     <row r="6">
@@ -403,7 +403,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>110031357760</v>
+        <v>110054114061</v>
       </c>
     </row>
     <row r="7">
@@ -411,7 +411,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>110041393989</v>
+        <v>110031411719</v>
       </c>
     </row>
     <row r="8">
@@ -419,7 +419,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>110038278887</v>
+        <v>110041513957</v>
       </c>
     </row>
     <row r="9">
@@ -427,7 +427,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>110070272151</v>
+        <v>110038511820</v>
       </c>
     </row>
     <row r="10">
@@ -435,7 +435,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>110070311984</v>
+        <v>110070272516</v>
       </c>
     </row>
     <row r="11">
@@ -443,7 +443,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>110044258638</v>
+        <v>110070312330</v>
       </c>
     </row>
   </sheetData>

</xml_diff>